<commit_message>
feat: add cubic model as a design and analysis option
</commit_message>
<xml_diff>
--- a/exemplos/ensaios-em-branco.xlsx
+++ b/exemplos/ensaios-em-branco.xlsx
@@ -755,7 +755,7 @@
         <v>Gerado em</v>
       </c>
       <c r="B5" t="str">
-        <v>17/08/2026, 17:34:46</v>
+        <v>11/09/2026, 11:28:58</v>
       </c>
     </row>
     <row r="7">
@@ -924,7 +924,7 @@
         <v>dados0</v>
       </c>
       <c r="B4" t="str">
-        <v>{"versaoEsquema":1,"geradoEm":"2026-08-17T20:34:46.533Z","experimento":{"nome":"Síntese do acetato de etila","grupo":"3"},"resposta":{"objetivo":"maximizar","nome":"Rendimento","unidade":"%"},"fatores":[{"nome":"Temperatura","unidade":"°C","min":50,"max":80,"casasDecimais":1,"centro":65,"semiAmplitude":15,"unidadeCodificada":15},{"nome":"Concentração do catalisador","unidade":"mol/L","min":0.05,"max":0.25,"casasDecimais":3,"centro":0.15,"semiAmplitude":0.1,"unidadeCodificada":0.1}],"config":{"tipoAlpha":"face","pontosCentrais":3,"limitMode":"absoluto","aleatorizar":true,"confianca":0.95,"alpha":1,"semente":3088485294,"k":2},"ensaios":[{"id":"E01","ordemPadrao":1,"ordemExecucao":1,"tipo":"fatorial","codificadosPlanejados":[-1,-1],"reais":[50,0.05],"resposta":null},{"id":"E02","ordemPadrao":2,"ordemExecucao":3,"tipo":"fatorial","codificadosPlanejados":[1,-1],"reais":[80,0.05],"resposta":null},{"id":"E03","ordemPadrao":3,"ordemExecucao":6,"tipo":"fatorial","codificadosPlanejados":[-1,1],"reais":[50,0.25],"resposta":null},{"id":"E04","ordemPadrao":4,"ordemExecucao":4,"tipo":"fatorial","codificadosPlanejados":[1,1],"reais":[80,0.25],"resposta":null},{"id":"E05","ordemPadrao":5,"ordemExecucao":5,"tipo":"axial","codificadosPlanejados":[-1,0],"reais":[50,0.15],"resposta":null},{"id":"E06","ordemPadrao":6,"ordemExecucao":10,"tipo":"axial","codificadosPlanejados":[1,0],"reais":[80,0.15],"resposta":null},{"id":"E07","ordemPadrao":7,"ordemExecucao":2,"tipo":"axial","codificadosPlanejados":[0,-1],"reais":[65,0.05],"resposta":null},{"id":"E08","ordemPadrao":8,"ordemExecucao":7,"tipo":"axial","codificadosPlanejados":[0,1],"reais":[65,0.25],"resposta":null},{"id":"E09","ordemPadrao":9,"ordemExecucao":11,"tipo":"central","codificadosPlanejados":[0,0],"reais":[65,0.15],"resposta":null},{"id":"E10","ordemPadrao":10,"ordemExecucao":8,"tipo":"central","codificadosPlanejados":[0,0],"reais":[65,0.15],"resposta":null},{"id":"E11","ordemPadrao":11,"ordemExecucao":9,"tipo":"central","codificadosPlanejados":[0,0],"reais":[65,0.15],"resposta":null}]}</v>
+        <v>{"versaoEsquema":1,"geradoEm":"2026-09-11T14:28:58.153Z","experimento":{"nome":"Síntese do acetato de etila","grupo":"3"},"resposta":{"objetivo":"maximizar","nome":"Rendimento","unidade":"%"},"fatores":[{"nome":"Temperatura","unidade":"°C","min":50,"max":80,"casasDecimais":1,"centro":65,"semiAmplitude":15,"unidadeCodificada":15},{"nome":"Concentração do catalisador","unidade":"mol/L","min":0.05,"max":0.25,"casasDecimais":3,"centro":0.15,"semiAmplitude":0.1,"unidadeCodificada":0.1}],"config":{"tipoAlpha":"face","pontosCentrais":3,"limitMode":"absoluto","aleatorizar":true,"confianca":0.95,"modelo":"quadratico","alpha":1,"semente":3088485294,"k":2},"ensaios":[{"id":"E01","ordemPadrao":1,"ordemExecucao":1,"tipo":"fatorial","codificadosPlanejados":[-1,-1],"reais":[50,0.05],"resposta":null},{"id":"E02","ordemPadrao":2,"ordemExecucao":3,"tipo":"fatorial","codificadosPlanejados":[1,-1],"reais":[80,0.05],"resposta":null},{"id":"E03","ordemPadrao":3,"ordemExecucao":6,"tipo":"fatorial","codificadosPlanejados":[-1,1],"reais":[50,0.25],"resposta":null},{"id":"E04","ordemPadrao":4,"ordemExecucao":4,"tipo":"fatorial","codificadosPlanejados":[1,1],"reais":[80,0.25],"resposta":null},{"id":"E05","ordemPadrao":5,"ordemExecucao":5,"tipo":"axial","codificadosPlanejados":[-1,0],"reais":[50,0.15],"resposta":null},{"id":"E06","ordemPadrao":6,"ordemExecucao":10,"tipo":"axial","codificadosPlanejados":[1,0],"reais":[80,0.15],"resposta":null},{"id":"E07","ordemPadrao":7,"ordemExecucao":2,"tipo":"axial","codificadosPlanejados":[0,-1],"reais":[65,0.05],"resposta":null},{"id":"E08","ordemPadrao":8,"ordemExecucao":7,"tipo":"axial","codificadosPlanejados":[0,1],"reais":[65,0.25],"resposta":null},{"id":"E09","ordemPadrao":9,"ordemExecucao":11,"tipo":"central","codificadosPlanejados":[0,0],"reais":[65,0.15],"resposta":null},{"id":"E10","ordemPadrao":10,"ordemExecucao":8,"tipo":"central","codificadosPlanejados":[0,0],"reais":[65,0.15],"resposta":null},{"id":"E11","ordemPadrao":11,"ordemExecucao":9,"tipo":"central","codificadosPlanejados":[0,0],"reais":[65,0.15],"resposta":null}]}</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(ui): redesign the site around a dashboard layout
</commit_message>
<xml_diff>
--- a/exemplos/ensaios-em-branco.xlsx
+++ b/exemplos/ensaios-em-branco.xlsx
@@ -405,14 +405,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:E12"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
     <col min="3" max="3" width="18.83203125" customWidth="1"/>
     <col min="4" max="4" width="18.83203125" customWidth="1"/>
     <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -431,9 +430,6 @@
       <c r="E1" t="str">
         <v>Rendimento (%)</v>
       </c>
-      <c r="F1" t="str">
-        <v>Observações</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="1">
@@ -448,9 +444,6 @@
       <c r="D2" s="3">
         <v>0.05</v>
       </c>
-      <c r="F2" t="str">
-        <v/>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="1">
@@ -465,9 +458,6 @@
       <c r="D3" s="3">
         <v>0.05</v>
       </c>
-      <c r="F3" t="str">
-        <v/>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="1">
@@ -482,9 +472,6 @@
       <c r="D4" s="3">
         <v>0.05</v>
       </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="1">
@@ -499,9 +486,6 @@
       <c r="D5" s="3">
         <v>0.25</v>
       </c>
-      <c r="F5" t="str">
-        <v/>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="1">
@@ -516,9 +500,6 @@
       <c r="D6" s="3">
         <v>0.15</v>
       </c>
-      <c r="F6" t="str">
-        <v/>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="1">
@@ -533,9 +514,6 @@
       <c r="D7" s="3">
         <v>0.25</v>
       </c>
-      <c r="F7" t="str">
-        <v/>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="1">
@@ -550,9 +528,6 @@
       <c r="D8" s="3">
         <v>0.25</v>
       </c>
-      <c r="F8" t="str">
-        <v/>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="1">
@@ -567,9 +542,6 @@
       <c r="D9" s="3">
         <v>0.15</v>
       </c>
-      <c r="F9" t="str">
-        <v/>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="1">
@@ -584,9 +556,6 @@
       <c r="D10" s="3">
         <v>0.15</v>
       </c>
-      <c r="F10" t="str">
-        <v/>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="1">
@@ -601,9 +570,6 @@
       <c r="D11" s="3">
         <v>0.15</v>
       </c>
-      <c r="F11" t="str">
-        <v/>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="1">
@@ -618,13 +584,10 @@
       <c r="D12" s="3">
         <v>0.15</v>
       </c>
-      <c r="F12" t="str">
-        <v/>
-      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -755,7 +718,7 @@
         <v>Gerado em</v>
       </c>
       <c r="B5" t="str">
-        <v>11/09/2026, 11:28:58</v>
+        <v>15/09/2026, 23:08:07</v>
       </c>
     </row>
     <row r="7">
@@ -924,7 +887,7 @@
         <v>dados0</v>
       </c>
       <c r="B4" t="str">
-        <v>{"versaoEsquema":1,"geradoEm":"2026-09-11T14:28:58.153Z","experimento":{"nome":"Síntese do acetato de etila","grupo":"3"},"resposta":{"objetivo":"maximizar","nome":"Rendimento","unidade":"%"},"fatores":[{"nome":"Temperatura","unidade":"°C","min":50,"max":80,"casasDecimais":1,"centro":65,"semiAmplitude":15,"unidadeCodificada":15},{"nome":"Concentração do catalisador","unidade":"mol/L","min":0.05,"max":0.25,"casasDecimais":3,"centro":0.15,"semiAmplitude":0.1,"unidadeCodificada":0.1}],"config":{"tipoAlpha":"face","pontosCentrais":3,"limitMode":"absoluto","aleatorizar":true,"confianca":0.95,"modelo":"quadratico","alpha":1,"semente":3088485294,"k":2},"ensaios":[{"id":"E01","ordemPadrao":1,"ordemExecucao":1,"tipo":"fatorial","codificadosPlanejados":[-1,-1],"reais":[50,0.05],"resposta":null},{"id":"E02","ordemPadrao":2,"ordemExecucao":3,"tipo":"fatorial","codificadosPlanejados":[1,-1],"reais":[80,0.05],"resposta":null},{"id":"E03","ordemPadrao":3,"ordemExecucao":6,"tipo":"fatorial","codificadosPlanejados":[-1,1],"reais":[50,0.25],"resposta":null},{"id":"E04","ordemPadrao":4,"ordemExecucao":4,"tipo":"fatorial","codificadosPlanejados":[1,1],"reais":[80,0.25],"resposta":null},{"id":"E05","ordemPadrao":5,"ordemExecucao":5,"tipo":"axial","codificadosPlanejados":[-1,0],"reais":[50,0.15],"resposta":null},{"id":"E06","ordemPadrao":6,"ordemExecucao":10,"tipo":"axial","codificadosPlanejados":[1,0],"reais":[80,0.15],"resposta":null},{"id":"E07","ordemPadrao":7,"ordemExecucao":2,"tipo":"axial","codificadosPlanejados":[0,-1],"reais":[65,0.05],"resposta":null},{"id":"E08","ordemPadrao":8,"ordemExecucao":7,"tipo":"axial","codificadosPlanejados":[0,1],"reais":[65,0.25],"resposta":null},{"id":"E09","ordemPadrao":9,"ordemExecucao":11,"tipo":"central","codificadosPlanejados":[0,0],"reais":[65,0.15],"resposta":null},{"id":"E10","ordemPadrao":10,"ordemExecucao":8,"tipo":"central","codificadosPlanejados":[0,0],"reais":[65,0.15],"resposta":null},{"id":"E11","ordemPadrao":11,"ordemExecucao":9,"tipo":"central","codificadosPlanejados":[0,0],"reais":[65,0.15],"resposta":null}]}</v>
+        <v>{"versaoEsquema":1,"geradoEm":"2026-09-16T02:08:07.054Z","experimento":{"nome":"Síntese do acetato de etila","grupo":"3"},"resposta":{"objetivo":"maximizar","nome":"Rendimento","unidade":"%"},"fatores":[{"nome":"Temperatura","unidade":"°C","min":50,"max":80,"casasDecimais":1,"centro":65,"semiAmplitude":15,"unidadeCodificada":15},{"nome":"Concentração do catalisador","unidade":"mol/L","min":0.05,"max":0.25,"casasDecimais":3,"centro":0.15,"semiAmplitude":0.1,"unidadeCodificada":0.1}],"config":{"tipoAlpha":"face","pontosCentrais":3,"limitMode":"absoluto","aleatorizar":true,"confianca":0.95,"modelo":"quadratico","alpha":1,"semente":3088485294,"k":2},"ensaios":[{"id":"E01","ordemPadrao":1,"ordemExecucao":1,"tipo":"fatorial","codificadosPlanejados":[-1,-1],"reais":[50,0.05],"resposta":null},{"id":"E02","ordemPadrao":2,"ordemExecucao":3,"tipo":"fatorial","codificadosPlanejados":[1,-1],"reais":[80,0.05],"resposta":null},{"id":"E03","ordemPadrao":3,"ordemExecucao":6,"tipo":"fatorial","codificadosPlanejados":[-1,1],"reais":[50,0.25],"resposta":null},{"id":"E04","ordemPadrao":4,"ordemExecucao":4,"tipo":"fatorial","codificadosPlanejados":[1,1],"reais":[80,0.25],"resposta":null},{"id":"E05","ordemPadrao":5,"ordemExecucao":5,"tipo":"axial","codificadosPlanejados":[-1,0],"reais":[50,0.15],"resposta":null},{"id":"E06","ordemPadrao":6,"ordemExecucao":10,"tipo":"axial","codificadosPlanejados":[1,0],"reais":[80,0.15],"resposta":null},{"id":"E07","ordemPadrao":7,"ordemExecucao":2,"tipo":"axial","codificadosPlanejados":[0,-1],"reais":[65,0.05],"resposta":null},{"id":"E08","ordemPadrao":8,"ordemExecucao":7,"tipo":"axial","codificadosPlanejados":[0,1],"reais":[65,0.25],"resposta":null},{"id":"E09","ordemPadrao":9,"ordemExecucao":11,"tipo":"central","codificadosPlanejados":[0,0],"reais":[65,0.15],"resposta":null},{"id":"E10","ordemPadrao":10,"ordemExecucao":8,"tipo":"central","codificadosPlanejados":[0,0],"reais":[65,0.15],"resposta":null},{"id":"E11","ordemPadrao":11,"ordemExecucao":9,"tipo":"central","codificadosPlanejados":[0,0],"reais":[65,0.15],"resposta":null}]}</v>
       </c>
     </row>
   </sheetData>

</xml_diff>